<commit_message>
Filtres Juin-Décembre 2026: mois S23-S53, simulation démarre Juin, Excel adaptés
</commit_message>
<xml_diff>
--- a/download/Modele_Suivi_Avancement_Gharb_2026.xlsx
+++ b/download/Modele_Suivi_Avancement_Gharb_2026.xlsx
@@ -551,7 +551,7 @@
     <row r="2" ht="32" customHeight="1">
       <c r="B2" s="1" t="inlineStr">
         <is>
-          <t>Suivi Physique et Financier des Projets — Région du Gharb 2026</t>
+          <t>Suivi Physique et Financier des Projets — Région du Gharb 2026 (Juin–Décembre)</t>
         </is>
       </c>
     </row>
@@ -4708,7 +4708,7 @@
     <row r="2" ht="32" customHeight="1">
       <c r="B2" s="1" t="inlineStr">
         <is>
-          <t>Récapitulatif par Province — Région du Gharb 2026</t>
+          <t>Récapitulatif par Province — Région du Gharb 2026 (Juin–Décembre)</t>
         </is>
       </c>
     </row>
@@ -4992,7 +4992,7 @@
     <row r="2" ht="32" customHeight="1">
       <c r="B2" s="1" t="inlineStr">
         <is>
-          <t>Récapitulatif par Secteur — Région du Gharb 2026</t>
+          <t>Récapitulatif par Secteur — Région du Gharb 2026 (Juin–Décembre)</t>
         </is>
       </c>
     </row>
@@ -5275,7 +5275,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:H35"/>
+  <dimension ref="A1:H35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -5292,11 +5292,12 @@
       </c>
     </row>
     <row r="3" ht="8" customHeight="1"/>
+    <row r="4"/>
     <row r="5">
       <c r="B5" s="15" t="inlineStr"/>
       <c r="C5" s="16" t="inlineStr">
         <is>
-          <t>Ce fichier Excel sert de modèle pour alimenter le dashboard SIG Gharb avec les données de suivi physique et financier des projets.</t>
+          <t>Ce fichier Excel sert de modèle pour alimenter le dashboard SIG Gharb avec les données de suivi physique et financier des projets (Juin à Décembre 2026).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Consultations négociées: société titulaire, dates ouverture/jugement/OSC, délai, réception + Excel adaptés
</commit_message>
<xml_diff>
--- a/download/Modele_Suivi_Avancement_Gharb_2026.xlsx
+++ b/download/Modele_Suivi_Avancement_Gharb_2026.xlsx
@@ -23,7 +23,7 @@
     <numFmt numFmtId="164" formatCode="0.0%"/>
     <numFmt numFmtId="165" formatCode="0.0"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -52,8 +52,14 @@
       <color rgb="001B2A4A"/>
       <sz val="11"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -80,8 +86,20 @@
         <fgColor rgb="00D6E0EB"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F4E79"/>
+        <bgColor rgb="001F4E79"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
+        <bgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="3">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -99,11 +117,17 @@
         <color rgb="00D6E0EB"/>
       </top>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -128,6 +152,12 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -525,7 +555,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:Q77"/>
+  <dimension ref="B2:X77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -637,6 +667,41 @@
           <t>Observations</t>
         </is>
       </c>
+      <c r="R4" s="18" t="inlineStr">
+        <is>
+          <t>N° Consultation</t>
+        </is>
+      </c>
+      <c r="S4" s="18" t="inlineStr">
+        <is>
+          <t>Société Titulaire</t>
+        </is>
+      </c>
+      <c r="T4" s="18" t="inlineStr">
+        <is>
+          <t>Date Ouverture Plis</t>
+        </is>
+      </c>
+      <c r="U4" s="18" t="inlineStr">
+        <is>
+          <t>Date Jugement</t>
+        </is>
+      </c>
+      <c r="V4" s="18" t="inlineStr">
+        <is>
+          <t>Date OSC</t>
+        </is>
+      </c>
+      <c r="W4" s="18" t="inlineStr">
+        <is>
+          <t>Délai Exécution (j)</t>
+        </is>
+      </c>
+      <c r="X4" s="18" t="inlineStr">
+        <is>
+          <t>Date Réception Provisoire</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="22" customHeight="1">
       <c r="B5" s="3" t="n">
@@ -692,6 +757,13 @@
       </c>
       <c r="P5" s="3" t="n"/>
       <c r="Q5" s="3" t="n"/>
+      <c r="R5" s="19" t="n"/>
+      <c r="S5" s="19" t="n"/>
+      <c r="T5" s="19" t="n"/>
+      <c r="U5" s="19" t="n"/>
+      <c r="V5" s="19" t="n"/>
+      <c r="W5" s="19" t="n"/>
+      <c r="X5" s="19" t="n"/>
     </row>
     <row r="6" ht="22" customHeight="1">
       <c r="B6" s="7" t="n">
@@ -747,6 +819,13 @@
       </c>
       <c r="P6" s="7" t="n"/>
       <c r="Q6" s="7" t="n"/>
+      <c r="R6" s="19" t="n"/>
+      <c r="S6" s="19" t="n"/>
+      <c r="T6" s="19" t="n"/>
+      <c r="U6" s="19" t="n"/>
+      <c r="V6" s="19" t="n"/>
+      <c r="W6" s="19" t="n"/>
+      <c r="X6" s="19" t="n"/>
     </row>
     <row r="7" ht="22" customHeight="1">
       <c r="B7" s="3" t="n">
@@ -802,6 +881,13 @@
       </c>
       <c r="P7" s="3" t="n"/>
       <c r="Q7" s="3" t="n"/>
+      <c r="R7" s="19" t="n"/>
+      <c r="S7" s="19" t="n"/>
+      <c r="T7" s="19" t="n"/>
+      <c r="U7" s="19" t="n"/>
+      <c r="V7" s="19" t="n"/>
+      <c r="W7" s="19" t="n"/>
+      <c r="X7" s="19" t="n"/>
     </row>
     <row r="8" ht="22" customHeight="1">
       <c r="B8" s="7" t="n">
@@ -857,6 +943,13 @@
       </c>
       <c r="P8" s="7" t="n"/>
       <c r="Q8" s="7" t="n"/>
+      <c r="R8" s="19" t="n"/>
+      <c r="S8" s="19" t="n"/>
+      <c r="T8" s="19" t="n"/>
+      <c r="U8" s="19" t="n"/>
+      <c r="V8" s="19" t="n"/>
+      <c r="W8" s="19" t="n"/>
+      <c r="X8" s="19" t="n"/>
     </row>
     <row r="9" ht="22" customHeight="1">
       <c r="B9" s="3" t="n">
@@ -912,6 +1005,13 @@
       </c>
       <c r="P9" s="3" t="n"/>
       <c r="Q9" s="3" t="n"/>
+      <c r="R9" s="19" t="n"/>
+      <c r="S9" s="19" t="n"/>
+      <c r="T9" s="19" t="n"/>
+      <c r="U9" s="19" t="n"/>
+      <c r="V9" s="19" t="n"/>
+      <c r="W9" s="19" t="n"/>
+      <c r="X9" s="19" t="n"/>
     </row>
     <row r="10" ht="22" customHeight="1">
       <c r="B10" s="7" t="n">
@@ -963,6 +1063,13 @@
       </c>
       <c r="P10" s="7" t="n"/>
       <c r="Q10" s="7" t="n"/>
+      <c r="R10" s="19" t="n"/>
+      <c r="S10" s="19" t="n"/>
+      <c r="T10" s="19" t="n"/>
+      <c r="U10" s="19" t="n"/>
+      <c r="V10" s="19" t="n"/>
+      <c r="W10" s="19" t="n"/>
+      <c r="X10" s="19" t="n"/>
     </row>
     <row r="11" ht="22" customHeight="1">
       <c r="B11" s="3" t="n">
@@ -1018,6 +1125,13 @@
       </c>
       <c r="P11" s="3" t="n"/>
       <c r="Q11" s="3" t="n"/>
+      <c r="R11" s="19" t="n"/>
+      <c r="S11" s="19" t="n"/>
+      <c r="T11" s="19" t="n"/>
+      <c r="U11" s="19" t="n"/>
+      <c r="V11" s="19" t="n"/>
+      <c r="W11" s="19" t="n"/>
+      <c r="X11" s="19" t="n"/>
     </row>
     <row r="12" ht="22" customHeight="1">
       <c r="B12" s="7" t="n">
@@ -1073,6 +1187,13 @@
       </c>
       <c r="P12" s="7" t="n"/>
       <c r="Q12" s="7" t="n"/>
+      <c r="R12" s="19" t="n"/>
+      <c r="S12" s="19" t="n"/>
+      <c r="T12" s="19" t="n"/>
+      <c r="U12" s="19" t="n"/>
+      <c r="V12" s="19" t="n"/>
+      <c r="W12" s="19" t="n"/>
+      <c r="X12" s="19" t="n"/>
     </row>
     <row r="13" ht="22" customHeight="1">
       <c r="B13" s="3" t="n">
@@ -1128,6 +1249,13 @@
       </c>
       <c r="P13" s="3" t="n"/>
       <c r="Q13" s="3" t="n"/>
+      <c r="R13" s="19" t="n"/>
+      <c r="S13" s="19" t="n"/>
+      <c r="T13" s="19" t="n"/>
+      <c r="U13" s="19" t="n"/>
+      <c r="V13" s="19" t="n"/>
+      <c r="W13" s="19" t="n"/>
+      <c r="X13" s="19" t="n"/>
     </row>
     <row r="14" ht="22" customHeight="1">
       <c r="B14" s="7" t="n">
@@ -1183,6 +1311,13 @@
       </c>
       <c r="P14" s="7" t="n"/>
       <c r="Q14" s="7" t="n"/>
+      <c r="R14" s="19" t="n"/>
+      <c r="S14" s="19" t="n"/>
+      <c r="T14" s="19" t="n"/>
+      <c r="U14" s="19" t="n"/>
+      <c r="V14" s="19" t="n"/>
+      <c r="W14" s="19" t="n"/>
+      <c r="X14" s="19" t="n"/>
     </row>
     <row r="15" ht="22" customHeight="1">
       <c r="B15" s="3" t="n">
@@ -1238,6 +1373,13 @@
       </c>
       <c r="P15" s="3" t="n"/>
       <c r="Q15" s="3" t="n"/>
+      <c r="R15" s="19" t="n"/>
+      <c r="S15" s="19" t="n"/>
+      <c r="T15" s="19" t="n"/>
+      <c r="U15" s="19" t="n"/>
+      <c r="V15" s="19" t="n"/>
+      <c r="W15" s="19" t="n"/>
+      <c r="X15" s="19" t="n"/>
     </row>
     <row r="16" ht="22" customHeight="1">
       <c r="B16" s="7" t="n">
@@ -1293,6 +1435,13 @@
       </c>
       <c r="P16" s="7" t="n"/>
       <c r="Q16" s="7" t="n"/>
+      <c r="R16" s="19" t="n"/>
+      <c r="S16" s="19" t="n"/>
+      <c r="T16" s="19" t="n"/>
+      <c r="U16" s="19" t="n"/>
+      <c r="V16" s="19" t="n"/>
+      <c r="W16" s="19" t="n"/>
+      <c r="X16" s="19" t="n"/>
     </row>
     <row r="17" ht="22" customHeight="1">
       <c r="B17" s="3" t="n">
@@ -1348,6 +1497,13 @@
       </c>
       <c r="P17" s="3" t="n"/>
       <c r="Q17" s="3" t="n"/>
+      <c r="R17" s="19" t="n"/>
+      <c r="S17" s="19" t="n"/>
+      <c r="T17" s="19" t="n"/>
+      <c r="U17" s="19" t="n"/>
+      <c r="V17" s="19" t="n"/>
+      <c r="W17" s="19" t="n"/>
+      <c r="X17" s="19" t="n"/>
     </row>
     <row r="18" ht="22" customHeight="1">
       <c r="B18" s="7" t="n">
@@ -1403,6 +1559,13 @@
       </c>
       <c r="P18" s="7" t="n"/>
       <c r="Q18" s="7" t="n"/>
+      <c r="R18" s="19" t="n"/>
+      <c r="S18" s="19" t="n"/>
+      <c r="T18" s="19" t="n"/>
+      <c r="U18" s="19" t="n"/>
+      <c r="V18" s="19" t="n"/>
+      <c r="W18" s="19" t="n"/>
+      <c r="X18" s="19" t="n"/>
     </row>
     <row r="19" ht="22" customHeight="1">
       <c r="B19" s="3" t="n">
@@ -1458,6 +1621,13 @@
       </c>
       <c r="P19" s="3" t="n"/>
       <c r="Q19" s="3" t="n"/>
+      <c r="R19" s="19" t="n"/>
+      <c r="S19" s="19" t="n"/>
+      <c r="T19" s="19" t="n"/>
+      <c r="U19" s="19" t="n"/>
+      <c r="V19" s="19" t="n"/>
+      <c r="W19" s="19" t="n"/>
+      <c r="X19" s="19" t="n"/>
     </row>
     <row r="20" ht="22" customHeight="1">
       <c r="B20" s="7" t="n">
@@ -1513,6 +1683,13 @@
       </c>
       <c r="P20" s="7" t="n"/>
       <c r="Q20" s="7" t="n"/>
+      <c r="R20" s="19" t="n"/>
+      <c r="S20" s="19" t="n"/>
+      <c r="T20" s="19" t="n"/>
+      <c r="U20" s="19" t="n"/>
+      <c r="V20" s="19" t="n"/>
+      <c r="W20" s="19" t="n"/>
+      <c r="X20" s="19" t="n"/>
     </row>
     <row r="21" ht="22" customHeight="1">
       <c r="B21" s="3" t="n">
@@ -1568,6 +1745,13 @@
       </c>
       <c r="P21" s="3" t="n"/>
       <c r="Q21" s="3" t="n"/>
+      <c r="R21" s="19" t="n"/>
+      <c r="S21" s="19" t="n"/>
+      <c r="T21" s="19" t="n"/>
+      <c r="U21" s="19" t="n"/>
+      <c r="V21" s="19" t="n"/>
+      <c r="W21" s="19" t="n"/>
+      <c r="X21" s="19" t="n"/>
     </row>
     <row r="22" ht="22" customHeight="1">
       <c r="B22" s="7" t="n">
@@ -1619,6 +1803,13 @@
       </c>
       <c r="P22" s="7" t="n"/>
       <c r="Q22" s="7" t="n"/>
+      <c r="R22" s="19" t="n"/>
+      <c r="S22" s="19" t="n"/>
+      <c r="T22" s="19" t="n"/>
+      <c r="U22" s="19" t="n"/>
+      <c r="V22" s="19" t="n"/>
+      <c r="W22" s="19" t="n"/>
+      <c r="X22" s="19" t="n"/>
     </row>
     <row r="23" ht="22" customHeight="1">
       <c r="B23" s="3" t="n">
@@ -1674,6 +1865,13 @@
       </c>
       <c r="P23" s="3" t="n"/>
       <c r="Q23" s="3" t="n"/>
+      <c r="R23" s="19" t="n"/>
+      <c r="S23" s="19" t="n"/>
+      <c r="T23" s="19" t="n"/>
+      <c r="U23" s="19" t="n"/>
+      <c r="V23" s="19" t="n"/>
+      <c r="W23" s="19" t="n"/>
+      <c r="X23" s="19" t="n"/>
     </row>
     <row r="24" ht="22" customHeight="1">
       <c r="B24" s="7" t="n">
@@ -1729,6 +1927,13 @@
       </c>
       <c r="P24" s="7" t="n"/>
       <c r="Q24" s="7" t="n"/>
+      <c r="R24" s="19" t="n"/>
+      <c r="S24" s="19" t="n"/>
+      <c r="T24" s="19" t="n"/>
+      <c r="U24" s="19" t="n"/>
+      <c r="V24" s="19" t="n"/>
+      <c r="W24" s="19" t="n"/>
+      <c r="X24" s="19" t="n"/>
     </row>
     <row r="25" ht="22" customHeight="1">
       <c r="B25" s="3" t="n">
@@ -1784,6 +1989,13 @@
       </c>
       <c r="P25" s="3" t="n"/>
       <c r="Q25" s="3" t="n"/>
+      <c r="R25" s="19" t="n"/>
+      <c r="S25" s="19" t="n"/>
+      <c r="T25" s="19" t="n"/>
+      <c r="U25" s="19" t="n"/>
+      <c r="V25" s="19" t="n"/>
+      <c r="W25" s="19" t="n"/>
+      <c r="X25" s="19" t="n"/>
     </row>
     <row r="26" ht="22" customHeight="1">
       <c r="B26" s="7" t="n">
@@ -1839,6 +2051,13 @@
       </c>
       <c r="P26" s="7" t="n"/>
       <c r="Q26" s="7" t="n"/>
+      <c r="R26" s="19" t="n"/>
+      <c r="S26" s="19" t="n"/>
+      <c r="T26" s="19" t="n"/>
+      <c r="U26" s="19" t="n"/>
+      <c r="V26" s="19" t="n"/>
+      <c r="W26" s="19" t="n"/>
+      <c r="X26" s="19" t="n"/>
     </row>
     <row r="27" ht="22" customHeight="1">
       <c r="B27" s="3" t="n">
@@ -1894,6 +2113,13 @@
       </c>
       <c r="P27" s="3" t="n"/>
       <c r="Q27" s="3" t="n"/>
+      <c r="R27" s="19" t="n"/>
+      <c r="S27" s="19" t="n"/>
+      <c r="T27" s="19" t="n"/>
+      <c r="U27" s="19" t="n"/>
+      <c r="V27" s="19" t="n"/>
+      <c r="W27" s="19" t="n"/>
+      <c r="X27" s="19" t="n"/>
     </row>
     <row r="28" ht="22" customHeight="1">
       <c r="B28" s="7" t="n">
@@ -1949,6 +2175,13 @@
       </c>
       <c r="P28" s="7" t="n"/>
       <c r="Q28" s="7" t="n"/>
+      <c r="R28" s="19" t="n"/>
+      <c r="S28" s="19" t="n"/>
+      <c r="T28" s="19" t="n"/>
+      <c r="U28" s="19" t="n"/>
+      <c r="V28" s="19" t="n"/>
+      <c r="W28" s="19" t="n"/>
+      <c r="X28" s="19" t="n"/>
     </row>
     <row r="29" ht="22" customHeight="1">
       <c r="B29" s="3" t="n">
@@ -2004,6 +2237,13 @@
       </c>
       <c r="P29" s="3" t="n"/>
       <c r="Q29" s="3" t="n"/>
+      <c r="R29" s="19" t="n"/>
+      <c r="S29" s="19" t="n"/>
+      <c r="T29" s="19" t="n"/>
+      <c r="U29" s="19" t="n"/>
+      <c r="V29" s="19" t="n"/>
+      <c r="W29" s="19" t="n"/>
+      <c r="X29" s="19" t="n"/>
     </row>
     <row r="30" ht="22" customHeight="1">
       <c r="B30" s="7" t="n">
@@ -2059,6 +2299,13 @@
       </c>
       <c r="P30" s="7" t="n"/>
       <c r="Q30" s="7" t="n"/>
+      <c r="R30" s="19" t="n"/>
+      <c r="S30" s="19" t="n"/>
+      <c r="T30" s="19" t="n"/>
+      <c r="U30" s="19" t="n"/>
+      <c r="V30" s="19" t="n"/>
+      <c r="W30" s="19" t="n"/>
+      <c r="X30" s="19" t="n"/>
     </row>
     <row r="31" ht="22" customHeight="1">
       <c r="B31" s="3" t="n">
@@ -2114,6 +2361,13 @@
       </c>
       <c r="P31" s="3" t="n"/>
       <c r="Q31" s="3" t="n"/>
+      <c r="R31" s="19" t="n"/>
+      <c r="S31" s="19" t="n"/>
+      <c r="T31" s="19" t="n"/>
+      <c r="U31" s="19" t="n"/>
+      <c r="V31" s="19" t="n"/>
+      <c r="W31" s="19" t="n"/>
+      <c r="X31" s="19" t="n"/>
     </row>
     <row r="32" ht="22" customHeight="1">
       <c r="B32" s="7" t="n">
@@ -2169,6 +2423,13 @@
       </c>
       <c r="P32" s="7" t="n"/>
       <c r="Q32" s="7" t="n"/>
+      <c r="R32" s="19" t="n"/>
+      <c r="S32" s="19" t="n"/>
+      <c r="T32" s="19" t="n"/>
+      <c r="U32" s="19" t="n"/>
+      <c r="V32" s="19" t="n"/>
+      <c r="W32" s="19" t="n"/>
+      <c r="X32" s="19" t="n"/>
     </row>
     <row r="33" ht="22" customHeight="1">
       <c r="B33" s="3" t="n">
@@ -2224,6 +2485,13 @@
       </c>
       <c r="P33" s="3" t="n"/>
       <c r="Q33" s="3" t="n"/>
+      <c r="R33" s="19" t="n"/>
+      <c r="S33" s="19" t="n"/>
+      <c r="T33" s="19" t="n"/>
+      <c r="U33" s="19" t="n"/>
+      <c r="V33" s="19" t="n"/>
+      <c r="W33" s="19" t="n"/>
+      <c r="X33" s="19" t="n"/>
     </row>
     <row r="34" ht="22" customHeight="1">
       <c r="B34" s="7" t="n">
@@ -2279,6 +2547,13 @@
       </c>
       <c r="P34" s="7" t="n"/>
       <c r="Q34" s="7" t="n"/>
+      <c r="R34" s="19" t="n"/>
+      <c r="S34" s="19" t="n"/>
+      <c r="T34" s="19" t="n"/>
+      <c r="U34" s="19" t="n"/>
+      <c r="V34" s="19" t="n"/>
+      <c r="W34" s="19" t="n"/>
+      <c r="X34" s="19" t="n"/>
     </row>
     <row r="35" ht="22" customHeight="1">
       <c r="B35" s="3" t="n">
@@ -2334,6 +2609,13 @@
       </c>
       <c r="P35" s="3" t="n"/>
       <c r="Q35" s="3" t="n"/>
+      <c r="R35" s="19" t="n"/>
+      <c r="S35" s="19" t="n"/>
+      <c r="T35" s="19" t="n"/>
+      <c r="U35" s="19" t="n"/>
+      <c r="V35" s="19" t="n"/>
+      <c r="W35" s="19" t="n"/>
+      <c r="X35" s="19" t="n"/>
     </row>
     <row r="36" ht="22" customHeight="1">
       <c r="B36" s="7" t="n">
@@ -2389,6 +2671,13 @@
       </c>
       <c r="P36" s="7" t="n"/>
       <c r="Q36" s="7" t="n"/>
+      <c r="R36" s="19" t="n"/>
+      <c r="S36" s="19" t="n"/>
+      <c r="T36" s="19" t="n"/>
+      <c r="U36" s="19" t="n"/>
+      <c r="V36" s="19" t="n"/>
+      <c r="W36" s="19" t="n"/>
+      <c r="X36" s="19" t="n"/>
     </row>
     <row r="37" ht="22" customHeight="1">
       <c r="B37" s="3" t="n">
@@ -2444,6 +2733,13 @@
       </c>
       <c r="P37" s="3" t="n"/>
       <c r="Q37" s="3" t="n"/>
+      <c r="R37" s="19" t="n"/>
+      <c r="S37" s="19" t="n"/>
+      <c r="T37" s="19" t="n"/>
+      <c r="U37" s="19" t="n"/>
+      <c r="V37" s="19" t="n"/>
+      <c r="W37" s="19" t="n"/>
+      <c r="X37" s="19" t="n"/>
     </row>
     <row r="38" ht="22" customHeight="1">
       <c r="B38" s="7" t="n">
@@ -2499,6 +2795,13 @@
       </c>
       <c r="P38" s="7" t="n"/>
       <c r="Q38" s="7" t="n"/>
+      <c r="R38" s="19" t="n"/>
+      <c r="S38" s="19" t="n"/>
+      <c r="T38" s="19" t="n"/>
+      <c r="U38" s="19" t="n"/>
+      <c r="V38" s="19" t="n"/>
+      <c r="W38" s="19" t="n"/>
+      <c r="X38" s="19" t="n"/>
     </row>
     <row r="39" ht="22" customHeight="1">
       <c r="B39" s="3" t="n">
@@ -2554,6 +2857,13 @@
       </c>
       <c r="P39" s="3" t="n"/>
       <c r="Q39" s="3" t="n"/>
+      <c r="R39" s="19" t="n"/>
+      <c r="S39" s="19" t="n"/>
+      <c r="T39" s="19" t="n"/>
+      <c r="U39" s="19" t="n"/>
+      <c r="V39" s="19" t="n"/>
+      <c r="W39" s="19" t="n"/>
+      <c r="X39" s="19" t="n"/>
     </row>
     <row r="40" ht="22" customHeight="1">
       <c r="B40" s="7" t="n">
@@ -2609,6 +2919,13 @@
       </c>
       <c r="P40" s="7" t="n"/>
       <c r="Q40" s="7" t="n"/>
+      <c r="R40" s="19" t="n"/>
+      <c r="S40" s="19" t="n"/>
+      <c r="T40" s="19" t="n"/>
+      <c r="U40" s="19" t="n"/>
+      <c r="V40" s="19" t="n"/>
+      <c r="W40" s="19" t="n"/>
+      <c r="X40" s="19" t="n"/>
     </row>
     <row r="41" ht="22" customHeight="1">
       <c r="B41" s="3" t="n">
@@ -2664,6 +2981,13 @@
       </c>
       <c r="P41" s="3" t="n"/>
       <c r="Q41" s="3" t="n"/>
+      <c r="R41" s="19" t="n"/>
+      <c r="S41" s="19" t="n"/>
+      <c r="T41" s="19" t="n"/>
+      <c r="U41" s="19" t="n"/>
+      <c r="V41" s="19" t="n"/>
+      <c r="W41" s="19" t="n"/>
+      <c r="X41" s="19" t="n"/>
     </row>
     <row r="42" ht="22" customHeight="1">
       <c r="B42" s="7" t="n">
@@ -2719,6 +3043,13 @@
       </c>
       <c r="P42" s="7" t="n"/>
       <c r="Q42" s="7" t="n"/>
+      <c r="R42" s="19" t="n"/>
+      <c r="S42" s="19" t="n"/>
+      <c r="T42" s="19" t="n"/>
+      <c r="U42" s="19" t="n"/>
+      <c r="V42" s="19" t="n"/>
+      <c r="W42" s="19" t="n"/>
+      <c r="X42" s="19" t="n"/>
     </row>
     <row r="43" ht="22" customHeight="1">
       <c r="B43" s="3" t="n">
@@ -2770,6 +3101,13 @@
       </c>
       <c r="P43" s="3" t="n"/>
       <c r="Q43" s="3" t="n"/>
+      <c r="R43" s="19" t="n"/>
+      <c r="S43" s="19" t="n"/>
+      <c r="T43" s="19" t="n"/>
+      <c r="U43" s="19" t="n"/>
+      <c r="V43" s="19" t="n"/>
+      <c r="W43" s="19" t="n"/>
+      <c r="X43" s="19" t="n"/>
     </row>
     <row r="44" ht="22" customHeight="1">
       <c r="B44" s="7" t="n">
@@ -2821,6 +3159,13 @@
       </c>
       <c r="P44" s="7" t="n"/>
       <c r="Q44" s="7" t="n"/>
+      <c r="R44" s="19" t="n"/>
+      <c r="S44" s="19" t="n"/>
+      <c r="T44" s="19" t="n"/>
+      <c r="U44" s="19" t="n"/>
+      <c r="V44" s="19" t="n"/>
+      <c r="W44" s="19" t="n"/>
+      <c r="X44" s="19" t="n"/>
     </row>
     <row r="45" ht="22" customHeight="1">
       <c r="B45" s="3" t="n">
@@ -2872,6 +3217,13 @@
       </c>
       <c r="P45" s="3" t="n"/>
       <c r="Q45" s="3" t="n"/>
+      <c r="R45" s="19" t="n"/>
+      <c r="S45" s="19" t="n"/>
+      <c r="T45" s="19" t="n"/>
+      <c r="U45" s="19" t="n"/>
+      <c r="V45" s="19" t="n"/>
+      <c r="W45" s="19" t="n"/>
+      <c r="X45" s="19" t="n"/>
     </row>
     <row r="46" ht="22" customHeight="1">
       <c r="B46" s="7" t="n">
@@ -2927,6 +3279,13 @@
       </c>
       <c r="P46" s="7" t="n"/>
       <c r="Q46" s="7" t="n"/>
+      <c r="R46" s="19" t="n"/>
+      <c r="S46" s="19" t="n"/>
+      <c r="T46" s="19" t="n"/>
+      <c r="U46" s="19" t="n"/>
+      <c r="V46" s="19" t="n"/>
+      <c r="W46" s="19" t="n"/>
+      <c r="X46" s="19" t="n"/>
     </row>
     <row r="47" ht="22" customHeight="1">
       <c r="B47" s="3" t="n">
@@ -2982,6 +3341,13 @@
       </c>
       <c r="P47" s="3" t="n"/>
       <c r="Q47" s="3" t="n"/>
+      <c r="R47" s="19" t="n"/>
+      <c r="S47" s="19" t="n"/>
+      <c r="T47" s="19" t="n"/>
+      <c r="U47" s="19" t="n"/>
+      <c r="V47" s="19" t="n"/>
+      <c r="W47" s="19" t="n"/>
+      <c r="X47" s="19" t="n"/>
     </row>
     <row r="48" ht="22" customHeight="1">
       <c r="B48" s="7" t="n">
@@ -3037,6 +3403,13 @@
       </c>
       <c r="P48" s="7" t="n"/>
       <c r="Q48" s="7" t="n"/>
+      <c r="R48" s="19" t="n"/>
+      <c r="S48" s="19" t="n"/>
+      <c r="T48" s="19" t="n"/>
+      <c r="U48" s="19" t="n"/>
+      <c r="V48" s="19" t="n"/>
+      <c r="W48" s="19" t="n"/>
+      <c r="X48" s="19" t="n"/>
     </row>
     <row r="49" ht="22" customHeight="1">
       <c r="B49" s="3" t="n">
@@ -3092,6 +3465,13 @@
       </c>
       <c r="P49" s="3" t="n"/>
       <c r="Q49" s="3" t="n"/>
+      <c r="R49" s="19" t="n"/>
+      <c r="S49" s="19" t="n"/>
+      <c r="T49" s="19" t="n"/>
+      <c r="U49" s="19" t="n"/>
+      <c r="V49" s="19" t="n"/>
+      <c r="W49" s="19" t="n"/>
+      <c r="X49" s="19" t="n"/>
     </row>
     <row r="50" ht="22" customHeight="1">
       <c r="B50" s="7" t="n">
@@ -3147,6 +3527,13 @@
       </c>
       <c r="P50" s="7" t="n"/>
       <c r="Q50" s="7" t="n"/>
+      <c r="R50" s="19" t="n"/>
+      <c r="S50" s="19" t="n"/>
+      <c r="T50" s="19" t="n"/>
+      <c r="U50" s="19" t="n"/>
+      <c r="V50" s="19" t="n"/>
+      <c r="W50" s="19" t="n"/>
+      <c r="X50" s="19" t="n"/>
     </row>
     <row r="51" ht="22" customHeight="1">
       <c r="B51" s="3" t="n">
@@ -3202,6 +3589,13 @@
       </c>
       <c r="P51" s="3" t="n"/>
       <c r="Q51" s="3" t="n"/>
+      <c r="R51" s="19" t="n"/>
+      <c r="S51" s="19" t="n"/>
+      <c r="T51" s="19" t="n"/>
+      <c r="U51" s="19" t="n"/>
+      <c r="V51" s="19" t="n"/>
+      <c r="W51" s="19" t="n"/>
+      <c r="X51" s="19" t="n"/>
     </row>
     <row r="52" ht="22" customHeight="1">
       <c r="B52" s="7" t="n">
@@ -3253,6 +3647,13 @@
       </c>
       <c r="P52" s="7" t="n"/>
       <c r="Q52" s="7" t="n"/>
+      <c r="R52" s="19" t="n"/>
+      <c r="S52" s="19" t="n"/>
+      <c r="T52" s="19" t="n"/>
+      <c r="U52" s="19" t="n"/>
+      <c r="V52" s="19" t="n"/>
+      <c r="W52" s="19" t="n"/>
+      <c r="X52" s="19" t="n"/>
     </row>
     <row r="53" ht="22" customHeight="1">
       <c r="B53" s="3" t="n">
@@ -3304,6 +3705,13 @@
       </c>
       <c r="P53" s="3" t="n"/>
       <c r="Q53" s="3" t="n"/>
+      <c r="R53" s="19" t="n"/>
+      <c r="S53" s="19" t="n"/>
+      <c r="T53" s="19" t="n"/>
+      <c r="U53" s="19" t="n"/>
+      <c r="V53" s="19" t="n"/>
+      <c r="W53" s="19" t="n"/>
+      <c r="X53" s="19" t="n"/>
     </row>
     <row r="54" ht="22" customHeight="1">
       <c r="B54" s="7" t="n">
@@ -3359,6 +3767,13 @@
       </c>
       <c r="P54" s="7" t="n"/>
       <c r="Q54" s="7" t="n"/>
+      <c r="R54" s="19" t="n"/>
+      <c r="S54" s="19" t="n"/>
+      <c r="T54" s="19" t="n"/>
+      <c r="U54" s="19" t="n"/>
+      <c r="V54" s="19" t="n"/>
+      <c r="W54" s="19" t="n"/>
+      <c r="X54" s="19" t="n"/>
     </row>
     <row r="55" ht="22" customHeight="1">
       <c r="B55" s="3" t="n">
@@ -3414,6 +3829,13 @@
       </c>
       <c r="P55" s="3" t="n"/>
       <c r="Q55" s="3" t="n"/>
+      <c r="R55" s="19" t="n"/>
+      <c r="S55" s="19" t="n"/>
+      <c r="T55" s="19" t="n"/>
+      <c r="U55" s="19" t="n"/>
+      <c r="V55" s="19" t="n"/>
+      <c r="W55" s="19" t="n"/>
+      <c r="X55" s="19" t="n"/>
     </row>
     <row r="56" ht="22" customHeight="1">
       <c r="B56" s="7" t="n">
@@ -3469,6 +3891,13 @@
       </c>
       <c r="P56" s="7" t="n"/>
       <c r="Q56" s="7" t="n"/>
+      <c r="R56" s="19" t="n"/>
+      <c r="S56" s="19" t="n"/>
+      <c r="T56" s="19" t="n"/>
+      <c r="U56" s="19" t="n"/>
+      <c r="V56" s="19" t="n"/>
+      <c r="W56" s="19" t="n"/>
+      <c r="X56" s="19" t="n"/>
     </row>
     <row r="57" ht="22" customHeight="1">
       <c r="B57" s="3" t="n">
@@ -3524,6 +3953,13 @@
       </c>
       <c r="P57" s="3" t="n"/>
       <c r="Q57" s="3" t="n"/>
+      <c r="R57" s="19" t="n"/>
+      <c r="S57" s="19" t="n"/>
+      <c r="T57" s="19" t="n"/>
+      <c r="U57" s="19" t="n"/>
+      <c r="V57" s="19" t="n"/>
+      <c r="W57" s="19" t="n"/>
+      <c r="X57" s="19" t="n"/>
     </row>
     <row r="58" ht="22" customHeight="1">
       <c r="B58" s="7" t="n">
@@ -3579,6 +4015,13 @@
       </c>
       <c r="P58" s="7" t="n"/>
       <c r="Q58" s="7" t="n"/>
+      <c r="R58" s="19" t="n"/>
+      <c r="S58" s="19" t="n"/>
+      <c r="T58" s="19" t="n"/>
+      <c r="U58" s="19" t="n"/>
+      <c r="V58" s="19" t="n"/>
+      <c r="W58" s="19" t="n"/>
+      <c r="X58" s="19" t="n"/>
     </row>
     <row r="59" ht="22" customHeight="1">
       <c r="B59" s="3" t="n">
@@ -3634,6 +4077,13 @@
       </c>
       <c r="P59" s="3" t="n"/>
       <c r="Q59" s="3" t="n"/>
+      <c r="R59" s="19" t="n"/>
+      <c r="S59" s="19" t="n"/>
+      <c r="T59" s="19" t="n"/>
+      <c r="U59" s="19" t="n"/>
+      <c r="V59" s="19" t="n"/>
+      <c r="W59" s="19" t="n"/>
+      <c r="X59" s="19" t="n"/>
     </row>
     <row r="60" ht="22" customHeight="1">
       <c r="B60" s="7" t="n">
@@ -3689,6 +4139,13 @@
       </c>
       <c r="P60" s="7" t="n"/>
       <c r="Q60" s="7" t="n"/>
+      <c r="R60" s="19" t="n"/>
+      <c r="S60" s="19" t="n"/>
+      <c r="T60" s="19" t="n"/>
+      <c r="U60" s="19" t="n"/>
+      <c r="V60" s="19" t="n"/>
+      <c r="W60" s="19" t="n"/>
+      <c r="X60" s="19" t="n"/>
     </row>
     <row r="61" ht="22" customHeight="1">
       <c r="B61" s="3" t="n">
@@ -3744,6 +4201,13 @@
       </c>
       <c r="P61" s="3" t="n"/>
       <c r="Q61" s="3" t="n"/>
+      <c r="R61" s="19" t="n"/>
+      <c r="S61" s="19" t="n"/>
+      <c r="T61" s="19" t="n"/>
+      <c r="U61" s="19" t="n"/>
+      <c r="V61" s="19" t="n"/>
+      <c r="W61" s="19" t="n"/>
+      <c r="X61" s="19" t="n"/>
     </row>
     <row r="62" ht="22" customHeight="1">
       <c r="B62" s="7" t="n">
@@ -3799,6 +4263,13 @@
       </c>
       <c r="P62" s="7" t="n"/>
       <c r="Q62" s="7" t="n"/>
+      <c r="R62" s="19" t="n"/>
+      <c r="S62" s="19" t="n"/>
+      <c r="T62" s="19" t="n"/>
+      <c r="U62" s="19" t="n"/>
+      <c r="V62" s="19" t="n"/>
+      <c r="W62" s="19" t="n"/>
+      <c r="X62" s="19" t="n"/>
     </row>
     <row r="63" ht="22" customHeight="1">
       <c r="B63" s="3" t="n">
@@ -3854,6 +4325,13 @@
       </c>
       <c r="P63" s="3" t="n"/>
       <c r="Q63" s="3" t="n"/>
+      <c r="R63" s="19" t="n"/>
+      <c r="S63" s="19" t="n"/>
+      <c r="T63" s="19" t="n"/>
+      <c r="U63" s="19" t="n"/>
+      <c r="V63" s="19" t="n"/>
+      <c r="W63" s="19" t="n"/>
+      <c r="X63" s="19" t="n"/>
     </row>
     <row r="64" ht="22" customHeight="1">
       <c r="B64" s="7" t="n">
@@ -3909,6 +4387,13 @@
       </c>
       <c r="P64" s="7" t="n"/>
       <c r="Q64" s="7" t="n"/>
+      <c r="R64" s="19" t="n"/>
+      <c r="S64" s="19" t="n"/>
+      <c r="T64" s="19" t="n"/>
+      <c r="U64" s="19" t="n"/>
+      <c r="V64" s="19" t="n"/>
+      <c r="W64" s="19" t="n"/>
+      <c r="X64" s="19" t="n"/>
     </row>
     <row r="65" ht="22" customHeight="1">
       <c r="B65" s="3" t="n">
@@ -3964,6 +4449,13 @@
       </c>
       <c r="P65" s="3" t="n"/>
       <c r="Q65" s="3" t="n"/>
+      <c r="R65" s="19" t="n"/>
+      <c r="S65" s="19" t="n"/>
+      <c r="T65" s="19" t="n"/>
+      <c r="U65" s="19" t="n"/>
+      <c r="V65" s="19" t="n"/>
+      <c r="W65" s="19" t="n"/>
+      <c r="X65" s="19" t="n"/>
     </row>
     <row r="66" ht="22" customHeight="1">
       <c r="B66" s="7" t="n">
@@ -4019,6 +4511,13 @@
       </c>
       <c r="P66" s="7" t="n"/>
       <c r="Q66" s="7" t="n"/>
+      <c r="R66" s="19" t="n"/>
+      <c r="S66" s="19" t="n"/>
+      <c r="T66" s="19" t="n"/>
+      <c r="U66" s="19" t="n"/>
+      <c r="V66" s="19" t="n"/>
+      <c r="W66" s="19" t="n"/>
+      <c r="X66" s="19" t="n"/>
     </row>
     <row r="67" ht="22" customHeight="1">
       <c r="B67" s="3" t="n">
@@ -4074,6 +4573,13 @@
       </c>
       <c r="P67" s="3" t="n"/>
       <c r="Q67" s="3" t="n"/>
+      <c r="R67" s="19" t="n"/>
+      <c r="S67" s="19" t="n"/>
+      <c r="T67" s="19" t="n"/>
+      <c r="U67" s="19" t="n"/>
+      <c r="V67" s="19" t="n"/>
+      <c r="W67" s="19" t="n"/>
+      <c r="X67" s="19" t="n"/>
     </row>
     <row r="68" ht="22" customHeight="1">
       <c r="B68" s="7" t="n">
@@ -4129,6 +4635,13 @@
       </c>
       <c r="P68" s="7" t="n"/>
       <c r="Q68" s="7" t="n"/>
+      <c r="R68" s="19" t="n"/>
+      <c r="S68" s="19" t="n"/>
+      <c r="T68" s="19" t="n"/>
+      <c r="U68" s="19" t="n"/>
+      <c r="V68" s="19" t="n"/>
+      <c r="W68" s="19" t="n"/>
+      <c r="X68" s="19" t="n"/>
     </row>
     <row r="69" ht="22" customHeight="1">
       <c r="B69" s="3" t="n">
@@ -4184,6 +4697,13 @@
       </c>
       <c r="P69" s="3" t="n"/>
       <c r="Q69" s="3" t="n"/>
+      <c r="R69" s="19" t="n"/>
+      <c r="S69" s="19" t="n"/>
+      <c r="T69" s="19" t="n"/>
+      <c r="U69" s="19" t="n"/>
+      <c r="V69" s="19" t="n"/>
+      <c r="W69" s="19" t="n"/>
+      <c r="X69" s="19" t="n"/>
     </row>
     <row r="70" ht="22" customHeight="1">
       <c r="B70" s="7" t="n">
@@ -4239,6 +4759,13 @@
       </c>
       <c r="P70" s="7" t="n"/>
       <c r="Q70" s="7" t="n"/>
+      <c r="R70" s="19" t="n"/>
+      <c r="S70" s="19" t="n"/>
+      <c r="T70" s="19" t="n"/>
+      <c r="U70" s="19" t="n"/>
+      <c r="V70" s="19" t="n"/>
+      <c r="W70" s="19" t="n"/>
+      <c r="X70" s="19" t="n"/>
     </row>
     <row r="71" ht="22" customHeight="1">
       <c r="B71" s="3" t="n">
@@ -4294,6 +4821,13 @@
       </c>
       <c r="P71" s="3" t="n"/>
       <c r="Q71" s="3" t="n"/>
+      <c r="R71" s="19" t="n"/>
+      <c r="S71" s="19" t="n"/>
+      <c r="T71" s="19" t="n"/>
+      <c r="U71" s="19" t="n"/>
+      <c r="V71" s="19" t="n"/>
+      <c r="W71" s="19" t="n"/>
+      <c r="X71" s="19" t="n"/>
     </row>
     <row r="72" ht="22" customHeight="1">
       <c r="B72" s="7" t="n">
@@ -4349,6 +4883,13 @@
       </c>
       <c r="P72" s="7" t="n"/>
       <c r="Q72" s="7" t="n"/>
+      <c r="R72" s="19" t="n"/>
+      <c r="S72" s="19" t="n"/>
+      <c r="T72" s="19" t="n"/>
+      <c r="U72" s="19" t="n"/>
+      <c r="V72" s="19" t="n"/>
+      <c r="W72" s="19" t="n"/>
+      <c r="X72" s="19" t="n"/>
     </row>
     <row r="73" ht="22" customHeight="1">
       <c r="B73" s="3" t="n">
@@ -4404,6 +4945,13 @@
       </c>
       <c r="P73" s="3" t="n"/>
       <c r="Q73" s="3" t="n"/>
+      <c r="R73" s="19" t="n"/>
+      <c r="S73" s="19" t="n"/>
+      <c r="T73" s="19" t="n"/>
+      <c r="U73" s="19" t="n"/>
+      <c r="V73" s="19" t="n"/>
+      <c r="W73" s="19" t="n"/>
+      <c r="X73" s="19" t="n"/>
     </row>
     <row r="74" ht="22" customHeight="1">
       <c r="B74" s="7" t="n">
@@ -4459,6 +5007,13 @@
       </c>
       <c r="P74" s="7" t="n"/>
       <c r="Q74" s="7" t="n"/>
+      <c r="R74" s="19" t="n"/>
+      <c r="S74" s="19" t="n"/>
+      <c r="T74" s="19" t="n"/>
+      <c r="U74" s="19" t="n"/>
+      <c r="V74" s="19" t="n"/>
+      <c r="W74" s="19" t="n"/>
+      <c r="X74" s="19" t="n"/>
     </row>
     <row r="75" ht="22" customHeight="1">
       <c r="B75" s="3" t="n">
@@ -4514,6 +5069,13 @@
       </c>
       <c r="P75" s="3" t="n"/>
       <c r="Q75" s="3" t="n"/>
+      <c r="R75" s="19" t="n"/>
+      <c r="S75" s="19" t="n"/>
+      <c r="T75" s="19" t="n"/>
+      <c r="U75" s="19" t="n"/>
+      <c r="V75" s="19" t="n"/>
+      <c r="W75" s="19" t="n"/>
+      <c r="X75" s="19" t="n"/>
     </row>
     <row r="76" ht="22" customHeight="1">
       <c r="B76" s="7" t="n">
@@ -4569,6 +5131,13 @@
       </c>
       <c r="P76" s="7" t="n"/>
       <c r="Q76" s="7" t="n"/>
+      <c r="R76" s="19" t="n"/>
+      <c r="S76" s="19" t="n"/>
+      <c r="T76" s="19" t="n"/>
+      <c r="U76" s="19" t="n"/>
+      <c r="V76" s="19" t="n"/>
+      <c r="W76" s="19" t="n"/>
+      <c r="X76" s="19" t="n"/>
     </row>
     <row r="77" ht="26" customHeight="1">
       <c r="B77" s="11" t="inlineStr">
@@ -5275,7 +5844,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H35"/>
+  <dimension ref="B2:H35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -5292,7 +5861,6 @@
       </c>
     </row>
     <row r="3" ht="8" customHeight="1"/>
-    <row r="4"/>
     <row r="5">
       <c r="B5" s="15" t="inlineStr"/>
       <c r="C5" s="16" t="inlineStr">

</xml_diff>